<commit_message>
Ajout d'un lien vers la page de Grant Dermody - Changement d'un morceau
</commit_message>
<xml_diff>
--- a/Liste_Partitions.xlsx
+++ b/Liste_Partitions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="175">
   <si>
     <t xml:space="preserve">titre</t>
   </si>
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Stand by me</t>
   </si>
   <si>
-    <t xml:space="preserve">Be. E.King</t>
+    <t xml:space="preserve">Ben E.King</t>
   </si>
   <si>
     <t xml:space="preserve">Soul</t>
@@ -421,7 +421,7 @@
     <t xml:space="preserve">video-score_Georgia_on_my_mind.mp4</t>
   </si>
   <si>
-    <t xml:space="preserve">Goodbye pork pie hat (diato)</t>
+    <t xml:space="preserve">Goodbye pork pie hat</t>
   </si>
   <si>
     <t xml:space="preserve">Charles Mingus</t>
@@ -430,16 +430,10 @@
     <t xml:space="preserve">Jazz / Blues</t>
   </si>
   <si>
-    <t xml:space="preserve">Goodbye pork pie hat Diato.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">video-score_Goodbye_pork_pie_hat__Charles_Mingus.mp4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goodbye pork pie hat (chroma)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goodbye pork pie hat Chroma.pdf</t>
+    <t xml:space="preserve">Goodbye pork pie hat Diato Chroma.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">video-score_goodbye-pork-pie-hat-charles-mingus.mp4</t>
   </si>
   <si>
     <t xml:space="preserve">Irish celtic music</t>
@@ -664,8 +658,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="20.85" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.85"/>
@@ -675,7 +669,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="7" style="1" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -695,7 +689,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -715,7 +709,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -735,7 +729,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -755,7 +749,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -775,7 +769,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -795,7 +789,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -815,7 +809,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>31</v>
       </c>
@@ -835,7 +829,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
@@ -855,7 +849,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
@@ -875,7 +869,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
@@ -895,7 +889,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
@@ -915,7 +909,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>52</v>
       </c>
@@ -935,7 +929,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>56</v>
       </c>
@@ -955,7 +949,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>60</v>
       </c>
@@ -975,7 +969,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
@@ -995,7 +989,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>68</v>
       </c>
@@ -1015,7 +1009,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>73</v>
       </c>
@@ -1035,7 +1029,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>77</v>
       </c>
@@ -1055,7 +1049,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>81</v>
       </c>
@@ -1075,7 +1069,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>84</v>
       </c>
@@ -1095,7 +1089,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>89</v>
       </c>
@@ -1115,7 +1109,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>93</v>
       </c>
@@ -1135,7 +1129,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>96</v>
       </c>
@@ -1152,7 +1146,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>99</v>
       </c>
@@ -1172,7 +1166,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>104</v>
       </c>
@@ -1192,7 +1186,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>107</v>
       </c>
@@ -1212,7 +1206,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>112</v>
       </c>
@@ -1232,7 +1226,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>116</v>
       </c>
@@ -1252,7 +1246,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
         <v>121</v>
       </c>
@@ -1272,7 +1266,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>125</v>
       </c>
@@ -1289,7 +1283,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>129</v>
       </c>
@@ -1309,7 +1303,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>133</v>
       </c>
@@ -1320,7 +1314,7 @@
         <v>135</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>136</v>
@@ -1329,223 +1323,206 @@
         <v>137</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>134</v>
+        <v>7</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>135</v>
+        <v>8</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F34" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>7</v>
+        <v>85</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>8</v>
+        <v>86</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>85</v>
+        <v>145</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>49</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>49</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C40" s="1" t="s">
+      <c r="E41" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D40" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="D42" s="1" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="20.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>171</v>
+        <v>7</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>62</v>
+        <v>13</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="G44" s="0"/>
+      <c r="G43" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
ajout de bobby casey
</commit_message>
<xml_diff>
--- a/Liste_Partitions.xlsx
+++ b/Liste_Partitions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="178">
   <si>
     <t xml:space="preserve">titre</t>
   </si>
@@ -545,6 +545,15 @@
   </si>
   <si>
     <t xml:space="preserve">video-score_The_red_river_valley.mp4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bobby Casey’s hornpipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bobby-caseys-hornpipe.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">video-score_bobby-caseys-hornpipe-public-domain.mp4</t>
   </si>
 </sst>
 </file>
@@ -658,7 +667,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="20.85" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.72"/>
@@ -1524,6 +1533,26 @@
       </c>
       <c r="G43" s="0"/>
     </row>
+    <row r="44" customFormat="false" ht="23.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>